<commit_message>
feat: separate editable closing base from financial publication
</commit_message>
<xml_diff>
--- a/e2e/fixtures/closing-v31-happy.xlsx
+++ b/e2e/fixtures/closing-v31-happy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V31_SOURCE" sheetId="1" r:id="Rb79781beda3c4ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V31_SOURCE" sheetId="1" r:id="R8bfe818290ed43e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="R$ #,##0.00"/>
+  <x:numFmts count="3">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0.00;[Red](#,##0.00)"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -37,27 +39,23 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF243B53"/>
+        <x:fgColor rgb="FF234E52"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="1">
     <x:border/>
-    <x:border>
-      <x:bottom style="double">
-        <x:color rgb="FF526D82"/>
-      </x:bottom>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -260,49 +258,49 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="22" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
         <x:v>reference</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="2" t="str">
         <x:v>amount</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="2" t="str">
         <x:v>date</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="2" t="str">
         <x:v>responsible</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" t="str">
-        <x:v>V31-001</x:v>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>SYNTHETIC-JULY-001</x:v>
       </x:c>
       <x:c r="B2" s="4" t="n">
         <x:v>125.5</x:v>
       </x:c>
-      <x:c r="C2" t="str">
-        <x:v>2026-09-05</x:v>
+      <x:c r="C2" s="5" t="n">
+        <x:v>46208</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>PARTICIPANT</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" t="str">
-        <x:v>V31-002</x:v>
+    <x:row r="3">
+      <x:c r="A3" s="3" t="str">
+        <x:v>SYNTHETIC-JULY-002</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
         <x:v>74.5</x:v>
       </x:c>
-      <x:c r="C3" t="str">
-        <x:v>2026-09-06</x:v>
+      <x:c r="C3" s="5" t="n">
+        <x:v>46209</x:v>
       </x:c>
       <x:c r="D3" t="str">
         <x:v>PARTICIPANT</x:v>

</xml_diff>